<commit_message>
update till end 2024
</commit_message>
<xml_diff>
--- a/DESTATIS_Data.xlsx
+++ b/DESTATIS_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timjascheck/Desktop/Quaterly-Output-Gap/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anatos91\Documents\Quaterly-Output-Gap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D19CD490-1DB2-CF42-BFCB-636817A1C316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0BF9BAD-1FE0-49B7-BBA4-B7AE1B66B91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4580" yWindow="2380" windowWidth="21600" windowHeight="11380" xr2:uid="{D91C66F5-F0F2-1148-A5B5-39C737905D32}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{D91C66F5-F0F2-1148-A5B5-39C737905D32}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -28,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
   <si>
     <t>preisbereinigt, verkettete Volumenang. (Mrd. EUR)</t>
   </si>
@@ -460,6 +458,15 @@
   </si>
   <si>
     <t>quarter</t>
+  </si>
+  <si>
+    <t>2024-Q2</t>
+  </si>
+  <si>
+    <t>2024-Q3</t>
+  </si>
+  <si>
+    <t>2024-Q4</t>
   </si>
 </sst>
 </file>
@@ -469,7 +476,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -547,8 +554,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -880,15 +887,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6775A59-AD61-FD4D-AEC5-5FE44EA4E70F}">
-  <dimension ref="A1:B134"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B137"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6328125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
         <v>140</v>
       </c>
@@ -896,7 +903,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -904,7 +911,7 @@
         <v>557.51700000000005</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -912,7 +919,7 @@
         <v>554.56600000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -920,7 +927,7 @@
         <v>553.35599999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -928,7 +935,7 @@
         <v>560.46799999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -936,7 +943,7 @@
         <v>569.05399999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -944,7 +951,7 @@
         <v>564.66600000000005</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -952,7 +959,7 @@
         <v>563.68299999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -960,7 +967,7 @@
         <v>561.86699999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -968,7 +975,7 @@
         <v>557.80100000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -976,7 +983,7 @@
         <v>557.649</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -984,7 +991,7 @@
         <v>560.90200000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -992,7 +999,7 @@
         <v>560.524</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -1000,7 +1007,7 @@
         <v>568.298</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -1008,7 +1015,7 @@
         <v>569.66</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -1016,7 +1023,7 @@
         <v>573.59400000000005</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -1024,7 +1031,7 @@
         <v>580.553</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1032,7 +1039,7 @@
         <v>578.47299999999996</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -1040,7 +1047,7 @@
         <v>582.71</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -1048,7 +1055,7 @@
         <v>583.76900000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1056,7 +1063,7 @@
         <v>583.99599999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -1064,7 +1071,7 @@
         <v>579.21100000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -1072,7 +1079,7 @@
         <v>587.07899999999995</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -1080,7 +1087,7 @@
         <v>589.04600000000005</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -1088,7 +1095,7 @@
         <v>593.43399999999997</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
@@ -1096,7 +1103,7 @@
         <v>590.351</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -1104,7 +1111,7 @@
         <v>597.99199999999996</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
@@ -1112,7 +1119,7 @@
         <v>599.80799999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
@@ -1120,7 +1127,7 @@
         <v>604.34699999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2">
       <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
@@ -1128,7 +1135,7 @@
         <v>609.98299999999995</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2">
       <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
@@ -1136,7 +1143,7 @@
         <v>607.41099999999994</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
@@ -1144,7 +1151,7 @@
         <v>610.28599999999994</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
@@ -1152,7 +1159,7 @@
         <v>607.78899999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2">
       <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
@@ -1160,7 +1167,7 @@
         <v>614.82500000000005</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2">
       <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
@@ -1168,7 +1175,7 @@
         <v>614.82500000000005</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
@@ -1176,7 +1183,7 @@
         <v>621.63400000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2">
       <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
@@ -1184,7 +1191,7 @@
         <v>626.77800000000002</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
@@ -1192,7 +1199,7 @@
         <v>635.72500000000002</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
@@ -1200,7 +1207,7 @@
         <v>640.86900000000003</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2">
       <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
@@ -1208,7 +1215,7 @@
         <v>640.56700000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
@@ -1216,7 +1223,7 @@
         <v>638.67499999999995</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
@@ -1224,7 +1231,7 @@
         <v>651.51800000000003</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
@@ -1232,7 +1239,7 @@
         <v>651.29100000000005</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
@@ -1240,7 +1247,7 @@
         <v>649.92899999999997</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
@@ -1248,7 +1255,7 @@
         <v>649.32399999999996</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
@@ -1256,7 +1263,7 @@
         <v>645.995</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
@@ -1264,7 +1271,7 @@
         <v>648.79399999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2">
       <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
@@ -1272,7 +1279,7 @@
         <v>651.971</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2">
       <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
@@ -1280,7 +1287,7 @@
         <v>651.06399999999996</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2">
       <c r="A50" s="2" t="s">
         <v>49</v>
       </c>
@@ -1288,7 +1295,7 @@
         <v>641.399</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2">
       <c r="A51" s="2" t="s">
         <v>50</v>
       </c>
@@ -1296,7 +1303,7 @@
         <v>642.08000000000004</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2">
       <c r="A52" s="2" t="s">
         <v>51</v>
       </c>
@@ -1304,7 +1311,7 @@
         <v>646.99699999999996</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2">
       <c r="A53" s="2" t="s">
         <v>52</v>
       </c>
@@ -1312,7 +1319,7 @@
         <v>648.81299999999999</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2">
       <c r="A54" s="2" t="s">
         <v>53</v>
       </c>
@@ -1320,7 +1327,7 @@
         <v>647.678</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2">
       <c r="A55" s="2" t="s">
         <v>54</v>
       </c>
@@ -1328,7 +1335,7 @@
         <v>651.00699999999995</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2">
       <c r="A56" s="2" t="s">
         <v>55</v>
       </c>
@@ -1336,7 +1343,7 @@
         <v>649.64499999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2">
       <c r="A57" s="2" t="s">
         <v>56</v>
       </c>
@@ -1344,7 +1351,7 @@
         <v>649.11599999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2">
       <c r="A58" s="2" t="s">
         <v>57</v>
       </c>
@@ -1352,7 +1359,7 @@
         <v>649.05899999999997</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2">
       <c r="A59" s="2" t="s">
         <v>58</v>
       </c>
@@ -1360,7 +1367,7 @@
         <v>652.53899999999999</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2">
       <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
@@ -1368,7 +1375,7 @@
         <v>658.06200000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2">
       <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
@@ -1376,7 +1383,7 @@
         <v>661.23900000000003</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2">
       <c r="A62" s="3" t="s">
         <v>61</v>
       </c>
@@ -1384,7 +1391,7 @@
         <v>667.65099999999995</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2">
       <c r="A63" s="3" t="s">
         <v>62</v>
       </c>
@@ -1392,7 +1399,7 @@
         <v>679.07500000000005</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:2">
       <c r="A64" s="3" t="s">
         <v>63</v>
       </c>
@@ -1400,7 +1407,7 @@
         <v>684.29499999999996</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:2">
       <c r="A65" s="3" t="s">
         <v>64</v>
       </c>
@@ -1408,7 +1415,7 @@
         <v>694.66</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
@@ -1416,7 +1423,7 @@
         <v>695.11400000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
@@ -1424,7 +1431,7 @@
         <v>701.01499999999999</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
@@ -1432,7 +1439,7 @@
         <v>704.57</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:2">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -1440,7 +1447,7 @@
         <v>709.11</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:2">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -1448,7 +1455,7 @@
         <v>713.649</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:2">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -1456,7 +1463,7 @@
         <v>711.98500000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:2">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
@@ -1464,7 +1471,7 @@
         <v>707.37</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -1472,7 +1479,7 @@
         <v>696.09699999999998</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -1480,7 +1487,7 @@
         <v>663.49</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:2">
       <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
@@ -1488,7 +1495,7 @@
         <v>664.54899999999998</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:2">
       <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
@@ -1496,7 +1503,7 @@
         <v>668.25599999999997</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:2">
       <c r="A77" s="2" t="s">
         <v>76</v>
       </c>
@@ -1504,7 +1511,7 @@
         <v>673.17399999999998</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:2">
       <c r="A78" s="2" t="s">
         <v>77</v>
       </c>
@@ -1512,7 +1519,7 @@
         <v>678.60199999999998</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:2">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -1520,7 +1527,7 @@
         <v>693.88400000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:2">
       <c r="A80" s="2" t="s">
         <v>79</v>
       </c>
@@ -1528,7 +1535,7 @@
         <v>699.63400000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:2">
       <c r="A81" s="2" t="s">
         <v>80</v>
       </c>
@@ -1536,7 +1543,7 @@
         <v>705.30799999999999</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:2">
       <c r="A82" s="2" t="s">
         <v>81</v>
       </c>
@@ -1544,7 +1551,7 @@
         <v>718.94500000000005</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:2">
       <c r="A83" s="2" t="s">
         <v>82</v>
       </c>
@@ -1552,7 +1559,7 @@
         <v>719.62599999999998</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:2">
       <c r="A84" s="2" t="s">
         <v>83</v>
       </c>
@@ -1560,7 +1567,7 @@
         <v>725.98099999999999</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:2">
       <c r="A85" s="2" t="s">
         <v>84</v>
       </c>
@@ -1568,7 +1575,7 @@
         <v>723.71100000000001</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:2">
       <c r="A86" s="2" t="s">
         <v>85</v>
       </c>
@@ -1576,7 +1583,7 @@
         <v>725.3</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:2">
       <c r="A87" s="2" t="s">
         <v>86</v>
       </c>
@@ -1584,7 +1591,7 @@
         <v>726.66099999999994</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:2">
       <c r="A88" s="2" t="s">
         <v>87</v>
       </c>
@@ -1592,7 +1599,7 @@
         <v>728.78</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:2">
       <c r="A89" s="2" t="s">
         <v>88</v>
       </c>
@@ -1600,7 +1607,7 @@
         <v>725.375</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:2">
       <c r="A90" s="2" t="s">
         <v>89</v>
       </c>
@@ -1608,7 +1615,7 @@
         <v>722.10400000000004</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:2">
       <c r="A91" s="2" t="s">
         <v>90</v>
       </c>
@@ -1616,7 +1623,7 @@
         <v>729.971</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:2">
       <c r="A92" s="2" t="s">
         <v>91</v>
       </c>
@@ -1624,7 +1631,7 @@
         <v>733.98099999999999</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:2">
       <c r="A93" s="2" t="s">
         <v>92</v>
       </c>
@@ -1632,7 +1639,7 @@
         <v>736.024</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:2">
       <c r="A94" s="2" t="s">
         <v>93</v>
       </c>
@@ -1640,7 +1647,7 @@
         <v>743.23</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:2">
       <c r="A95" s="2" t="s">
         <v>94</v>
       </c>
@@ -1648,7 +1655,7 @@
         <v>743.38099999999997</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:2">
       <c r="A96" s="2" t="s">
         <v>95</v>
       </c>
@@ -1656,7 +1663,7 @@
         <v>746.93700000000001</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:2">
       <c r="A97" s="2" t="s">
         <v>96</v>
       </c>
@@ -1664,7 +1671,7 @@
         <v>752.98900000000003</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:2">
       <c r="A98" s="2" t="s">
         <v>97</v>
       </c>
@@ -1672,7 +1679,7 @@
         <v>749.20699999999999</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:2">
       <c r="A99" s="2" t="s">
         <v>98</v>
       </c>
@@ -1680,7 +1687,7 @@
         <v>755.03200000000004</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:2">
       <c r="A100" s="2" t="s">
         <v>99</v>
       </c>
@@ -1688,7 +1695,7 @@
         <v>757.98199999999997</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:2">
       <c r="A101" s="2" t="s">
         <v>100</v>
       </c>
@@ -1696,7 +1703,7 @@
         <v>761.38699999999994</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:2">
       <c r="A102" s="2" t="s">
         <v>101</v>
       </c>
@@ -1704,7 +1711,7 @@
         <v>767.81799999999998</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:2">
       <c r="A103" s="2" t="s">
         <v>102</v>
       </c>
@@ -1712,7 +1719,7 @@
         <v>771.52499999999998</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:2">
       <c r="A104" s="2" t="s">
         <v>103</v>
       </c>
@@ -1720,7 +1727,7 @@
         <v>773.03800000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:2">
       <c r="A105" s="2" t="s">
         <v>104</v>
       </c>
@@ -1728,7 +1735,7 @@
         <v>775.98800000000006</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:2">
       <c r="A106" s="2" t="s">
         <v>105</v>
       </c>
@@ -1736,7 +1743,7 @@
         <v>785.29399999999998</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:2">
       <c r="A107" s="2" t="s">
         <v>106</v>
       </c>
@@ -1744,7 +1751,7 @@
         <v>792.55700000000002</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:2">
       <c r="A108" s="2" t="s">
         <v>107</v>
       </c>
@@ -1752,7 +1759,7 @@
         <v>797.55</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:2">
       <c r="A109" s="2" t="s">
         <v>108</v>
       </c>
@@ -1760,7 +1767,7 @@
         <v>805.11500000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:2">
       <c r="A110" s="2" t="s">
         <v>109</v>
       </c>
@@ -1768,7 +1775,7 @@
         <v>800.25400000000002</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:2">
       <c r="A111" s="2" t="s">
         <v>110</v>
       </c>
@@ -1776,7 +1783,7 @@
         <v>806.76099999999997</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:2">
       <c r="A112" s="2" t="s">
         <v>111</v>
       </c>
@@ -1784,7 +1791,7 @@
         <v>799.27099999999996</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:2">
       <c r="A113" s="2" t="s">
         <v>112</v>
       </c>
@@ -1792,7 +1799,7 @@
         <v>806.15499999999997</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:2">
       <c r="A114" s="2" t="s">
         <v>113</v>
       </c>
@@ -1800,7 +1807,7 @@
         <v>811.678</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:2">
       <c r="A115" s="2" t="s">
         <v>114</v>
       </c>
@@ -1808,7 +1815,7 @@
         <v>811.37599999999998</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:2">
       <c r="A116" s="2" t="s">
         <v>115</v>
       </c>
@@ -1816,7 +1823,7 @@
         <v>811.22400000000005</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:2">
       <c r="A117" s="2" t="s">
         <v>116</v>
       </c>
@@ -1824,7 +1831,7 @@
         <v>813.64499999999998</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:2">
       <c r="A118" s="2" t="s">
         <v>117</v>
       </c>
@@ -1832,7 +1839,7 @@
         <v>799.27</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:2">
       <c r="A119" s="2" t="s">
         <v>118</v>
       </c>
@@ -1840,7 +1847,7 @@
         <v>725.58500000000004</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:2">
       <c r="A120" s="2" t="s">
         <v>119</v>
       </c>
@@ -1848,7 +1855,7 @@
         <v>790.26800000000003</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:2">
       <c r="A121" s="2" t="s">
         <v>120</v>
       </c>
@@ -1856,7 +1863,7 @@
         <v>796.471</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:2">
       <c r="A122" s="2" t="s">
         <v>121</v>
       </c>
@@ -1864,7 +1871,7 @@
         <v>786.33399999999995</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:2">
       <c r="A123" s="2" t="s">
         <v>122</v>
       </c>
@@ -1872,7 +1879,7 @@
         <v>803.88599999999997</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:2">
       <c r="A124" s="2" t="s">
         <v>123</v>
       </c>
@@ -1880,7 +1887,7 @@
         <v>809.25699999999995</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:2">
       <c r="A125" s="2" t="s">
         <v>124</v>
       </c>
@@ -1888,7 +1895,7 @@
         <v>809.33299999999997</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:2">
       <c r="A126" s="2" t="s">
         <v>125</v>
       </c>
@@ -1896,7 +1903,7 @@
         <v>817.447</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:2">
       <c r="A127" s="2" t="s">
         <v>126</v>
       </c>
@@ -1904,7 +1911,7 @@
         <v>816.38800000000003</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:2">
       <c r="A128" s="2" t="s">
         <v>127</v>
       </c>
@@ -1912,7 +1919,7 @@
         <v>819.33799999999997</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:2">
       <c r="A129" s="2" t="s">
         <v>128</v>
       </c>
@@ -1920,7 +1927,7 @@
         <v>816.00900000000001</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:2">
       <c r="A130" s="2" t="s">
         <v>129</v>
       </c>
@@ -1928,7 +1935,7 @@
         <v>818.22199999999998</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:2">
       <c r="A131" s="2" t="s">
         <v>130</v>
       </c>
@@ -1936,7 +1943,7 @@
         <v>817.61699999999996</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:2">
       <c r="A132" s="2" t="s">
         <v>131</v>
       </c>
@@ -1944,7 +1951,7 @@
         <v>818.75199999999995</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:2">
       <c r="A133" s="2" t="s">
         <v>132</v>
       </c>
@@ -1952,12 +1959,36 @@
         <v>814.66700000000003</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:2">
       <c r="A134" s="2" t="s">
         <v>133</v>
       </c>
       <c r="B134" s="6">
         <v>816.40700000000004</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B135" s="5">
+        <v>813.89859999999999</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B136" s="5">
+        <v>814.75490000000002</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B137" s="5">
+        <v>813.12009999999998</v>
       </c>
     </row>
   </sheetData>
@@ -1968,34 +1999,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5343AA66-B0BD-8C41-8768-F5A8A3149688}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="15.6">
       <c r="A1" s="7" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
         <v>137</v>
       </c>

</xml_diff>